<commit_message>
Updated content from revision
</commit_message>
<xml_diff>
--- a/Data/GeoMx (protein)/Protein_panels_list.xlsx
+++ b/Data/GeoMx (protein)/Protein_panels_list.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://regionh-my.sharepoint.com/personal/vladyslav_vadymovych_tkach_regionh_dk2/Documents/PhD/Articles/First Article - Regional Microglial Reactivity/Data/GeoMx (protein)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://regionh-my.sharepoint.com/personal/vladyslav_vadymovych_tkach_regionh_dk2/Documents/PhD/Articles/Acta neuropathologica/Updated github/Data/GeoMx (protein)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="265" documentId="8_{4EA93997-FF3F-47A6-B117-87C4FE799FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FCA9226-503F-4AEE-B29C-310FB6FDDBE8}"/>
+  <xr:revisionPtr revIDLastSave="337" documentId="8_{4EA93997-FF3F-47A6-B117-87C4FE799FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7CBE4C1-9C96-40EA-9653-961D63EF5B52}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Protein_panel" sheetId="1" r:id="rId1"/>
+    <sheet name="Protein_panel_of_interest" sheetId="1" r:id="rId1"/>
     <sheet name="Full Panel" sheetId="4" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" refMode="R1C1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="152">
   <si>
     <t>Protein Name</t>
   </si>
@@ -330,13 +330,160 @@
   </si>
   <si>
     <t>C-type lectin domain containing 7A</t>
+  </si>
+  <si>
+    <t>GFAP</t>
+  </si>
+  <si>
+    <t>P14136, K7EMP8, A7REI1</t>
+  </si>
+  <si>
+    <t>glial fibrillary acidic protein</t>
+  </si>
+  <si>
+    <t>Astrocyte; Inflammation</t>
+  </si>
+  <si>
+    <t>MAP2</t>
+  </si>
+  <si>
+    <t>A0A024R409, A0A024R407, P11137, A0A024R3Z1, Q6NYC5, A0A024R3Y8</t>
+  </si>
+  <si>
+    <t>microtubule associated protein 2</t>
+  </si>
+  <si>
+    <t>Myelin basic protein</t>
+  </si>
+  <si>
+    <t>MBP</t>
+  </si>
+  <si>
+    <t>A0A024R384, P02686</t>
+  </si>
+  <si>
+    <t>myelin basic protein</t>
+  </si>
+  <si>
+    <t>Oligodendrocytes</t>
+  </si>
+  <si>
+    <t>NeuN</t>
+  </si>
+  <si>
+    <t>RBFOX3</t>
+  </si>
+  <si>
+    <t>A6NFN3</t>
+  </si>
+  <si>
+    <t>RNA binding fox-1 homolog 3</t>
+  </si>
+  <si>
+    <t>Neuron</t>
+  </si>
+  <si>
+    <t>Neurofilament light</t>
+  </si>
+  <si>
+    <t>NEFL</t>
+  </si>
+  <si>
+    <t>P07196</t>
+  </si>
+  <si>
+    <t>neurofilament light chain</t>
+  </si>
+  <si>
+    <t>S100B</t>
+  </si>
+  <si>
+    <t>A0A0S2Z4C5, P04271</t>
+  </si>
+  <si>
+    <t>S100 calcium binding protein B</t>
+  </si>
+  <si>
+    <t>Synaptophysin</t>
+  </si>
+  <si>
+    <t>SYP</t>
+  </si>
+  <si>
+    <t>P08247</t>
+  </si>
+  <si>
+    <t>synaptophysin</t>
+  </si>
+  <si>
+    <t>Synaptic Vesicle</t>
+  </si>
+  <si>
+    <t>Cytoskeleton; Neuron</t>
+  </si>
+  <si>
+    <t>Antigen; Astrocyte; Inflammation; Melanoma; Tumor</t>
+  </si>
+  <si>
+    <t>C4B</t>
+  </si>
+  <si>
+    <t>P0C0L4, P0C0L5</t>
+  </si>
+  <si>
+    <t>complement C4B (Chido blood group)</t>
+  </si>
+  <si>
+    <t>Astrocyte Activation</t>
+  </si>
+  <si>
+    <t>Vimentin</t>
+  </si>
+  <si>
+    <t>VIM</t>
+  </si>
+  <si>
+    <t>V9HWE1, P08670</t>
+  </si>
+  <si>
+    <t>vimentin</t>
+  </si>
+  <si>
+    <t>Astrocyte</t>
+  </si>
+  <si>
+    <t>EMP1</t>
+  </si>
+  <si>
+    <t>P54849, A0A024RAT0</t>
+  </si>
+  <si>
+    <t>epithelial membrane protein 1</t>
+  </si>
+  <si>
+    <t>A2 Astrocyte; Astrocyte</t>
+  </si>
+  <si>
+    <t>Olig2</t>
+  </si>
+  <si>
+    <t>OLIG2</t>
+  </si>
+  <si>
+    <t>Q13516</t>
+  </si>
+  <si>
+    <t>oligodendrocyte transcription factor 2</t>
+  </si>
+  <si>
+    <t>Proteins in grey are not related to microglia.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -467,6 +614,13 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.34998626667073579"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -833,7 +987,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -855,6 +1009,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Farve1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -914,9 +1070,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022 Tema">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -954,7 +1110,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1060,7 +1216,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1202,7 +1358,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1527,10 +1683,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7669E140-C99A-412D-A7C4-677A788C8819}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.140625" customWidth="1"/>
+    <col min="1" max="1" width="49.28515625" customWidth="1"/>
     <col min="2" max="2" width="30.42578125" customWidth="1"/>
     <col min="3" max="3" width="48.42578125" customWidth="1"/>
     <col min="4" max="4" width="19.42578125" customWidth="1"/>
@@ -1831,7 +1987,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>80</v>
       </c>
@@ -1851,7 +2007,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -1871,7 +2027,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>80</v>
       </c>
@@ -1891,144 +2047,383 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>55</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B28" t="s">
         <v>56</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C28" t="s">
         <v>96</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D28" t="s">
         <v>56</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E28" t="s">
         <v>57</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F28" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>55</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B29" t="s">
         <v>59</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C29" t="s">
         <v>97</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D29" t="s">
         <v>59</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E29" t="s">
         <v>60</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F29" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>55</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B30" t="s">
         <v>61</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C30" t="s">
         <v>98</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D30" t="s">
         <v>61</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E30" t="s">
         <v>62</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F30" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>55</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B31" t="s">
         <v>63</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C31" t="s">
         <v>99</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D31" t="s">
         <v>63</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E31" t="s">
         <v>64</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F31" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>55</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B32" t="s">
         <v>65</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C32" t="s">
         <v>100</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D32" t="s">
         <v>65</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E32" t="s">
         <v>66</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F32" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>55</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B33" t="s">
         <v>67</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C33" t="s">
         <v>101</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D33" t="s">
         <v>68</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E33" t="s">
         <v>69</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F33" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>55</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B34" t="s">
         <v>71</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C34" t="s">
         <v>102</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D34" t="s">
         <v>71</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E34" t="s">
         <v>72</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F34" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="10" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>